<commit_message>
feat: establish Planify Excel generation foundation
</commit_message>
<xml_diff>
--- a/output/finance_personal_2026_dark.xlsx
+++ b/output/finance_personal_2026_dark.xlsx
@@ -12,12 +12,17 @@
     <sheet name="Lançamentos" sheetId="3" r:id="rId3"/>
     <sheet name="Configurações" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="lista_cartoes">tblCartoes[Cartão]</definedName>
+    <definedName name="lista_categorias">tblCategorias[Categoria]</definedName>
+    <definedName name="lista_contas">tblContas[Conta]</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
   <si>
     <t>Bem-vindo ao Financeiro Pessoal</t>
   </si>
@@ -52,10 +57,19 @@
     <t>Saldo Disponível Hoje</t>
   </si>
   <si>
+    <t>SUMIFS(tblLancamentos[Valor],tblLancamentos[Tipo],"Receita")-SUMIFS(tblLancamentos[Valor],tblLancamentos[Tipo],"Despesa")</t>
+  </si>
+  <si>
     <t>Receitas do Mês</t>
   </si>
   <si>
+    <t>SUMIFS(tblLancamentos[Valor],tblLancamentos[Tipo],"Receita")</t>
+  </si>
+  <si>
     <t>Despesas do Mês</t>
+  </si>
+  <si>
+    <t>SUMIFS(tblLancamentos[Valor],tblLancamentos[Tipo],"Despesa")</t>
   </si>
   <si>
     <t>Lançamentos</t>
@@ -748,24 +762,21 @@
         <v>10</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="B5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5">
-      <c r="B5" s="7">
-        <f>=SUMIFS(tblLancamentos[Valor],tblLancamentos[Tipo],"Receita") - =SUMIFS(tblLancamentos[Valor],tblLancamentos[Tipo],"Despesa")</f>
-        <v>None</v>
-      </c>
-      <c r="D5" s="8">
-        <f>SUMIFS(tblLancamentos[Valor],tblLancamentos[Tipo],"Receita")</f>
-        <v>None</v>
-      </c>
-      <c r="E5" s="8">
-        <f>SUMIFS(tblLancamentos[Valor],tblLancamentos[Tipo],"Despesa")</f>
-        <v>None</v>
+      <c r="D5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -792,58 +803,57 @@
   <sheetData>
     <row r="2" spans="2:12">
       <c r="B2" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="2:12">
       <c r="B4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="H4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="J4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="K4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="L4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" formatCells="0" formatColumns="0" formatRows="0" insertRows="0" sort="0" autoFilter="0"/>
   <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor Inválido" error="Por favor, selecione um valor válido da lista." promptTitle="" prompt="" sqref="D5">
       <formula1>"Receita,Despesa,Transferência,Investimento,Resgate,Pagamento de dívida"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor Inválido" error="Por favor, selecione um valor válido da lista." promptTitle="" prompt="" sqref="E5">
-      <formula1>INDIRECT(tblCategorias[Categoria])</formula1>
+      <formula1>lista_categorias</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor Inválido" error="Por favor, selecione um valor válido da lista." promptTitle="" prompt="" sqref="F5">
-      <formula1>INDIRECT(tblContas[Conta])</formula1>
+      <formula1>lista_contas</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor Inválido" error="Por favor, selecione um valor válido da lista." promptTitle="" prompt="" sqref="G5">
-      <formula1>INDIRECT(tblCartoes[Cartão])</formula1>
+      <formula1>lista_cartoes</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor Inválido" error="Por favor, selecione um valor válido da lista." promptTitle="" prompt="" sqref="J5">
       <formula1>"Sim,Não"</formula1>
@@ -873,100 +883,100 @@
   <sheetData>
     <row r="2" spans="2:6">
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="2:6">
       <c r="B4" s="4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="2:6">
       <c r="B6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F6" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="2:6">
       <c r="B7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="2:6">
       <c r="B8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="2:6">
       <c r="B9" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="2:6">
       <c r="B10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="2:6">
       <c r="B11" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="2:6">
       <c r="B12" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="2:6">
       <c r="B13" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="2:6">
       <c r="B14" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="2:6">
       <c r="B15" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="2:6">
       <c r="B16" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="2:2">
       <c r="B17" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="2:2">
       <c r="B18" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="2:2">
       <c r="B19" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>